<commit_message>
PST-SSIS Test auto upload
</commit_message>
<xml_diff>
--- a/NINOX_Veranstaltungen_V01_20260211.xlsx
+++ b/NINOX_Veranstaltungen_V01_20260211.xlsx
@@ -749,7 +749,7 @@
       </c>
       <c r="AA3" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="AA4" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="AA5" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="AA6" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -1267,7 +1267,7 @@
       </c>
       <c r="AA7" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="AA8" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="AA9" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="AA10" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1755,7 @@
       </c>
       <c r="AA11" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1877,7 @@
       </c>
       <c r="AA12" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -1999,7 +1999,7 @@
       </c>
       <c r="AA13" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2136,7 @@
       </c>
       <c r="AA14" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="AA15" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2380,7 @@
       </c>
       <c r="AA16" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -2502,7 +2502,7 @@
       </c>
       <c r="AA17" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -2624,7 +2624,7 @@
       </c>
       <c r="AA18" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -2746,7 +2746,7 @@
       </c>
       <c r="AA19" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2868,7 @@
       </c>
       <c r="AA20" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -2995,7 +2995,7 @@
       </c>
       <c r="AA21" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -3122,7 +3122,7 @@
       </c>
       <c r="AA22" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -3249,7 +3249,7 @@
       </c>
       <c r="AA23" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -3376,7 +3376,7 @@
       </c>
       <c r="AA24" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -3493,7 +3493,7 @@
       </c>
       <c r="AA25" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -3610,7 +3610,7 @@
       </c>
       <c r="AA26" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -3727,7 +3727,7 @@
       </c>
       <c r="AA27" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -3844,7 +3844,7 @@
       </c>
       <c r="AA28" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -3961,7 +3961,7 @@
       </c>
       <c r="AA29" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -4078,7 +4078,7 @@
       </c>
       <c r="AA30" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -4200,7 +4200,7 @@
       </c>
       <c r="AA31" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -4337,7 +4337,7 @@
       </c>
       <c r="AA32" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -4474,7 +4474,7 @@
       </c>
       <c r="AA33" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="AA34" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -4748,7 +4748,7 @@
       </c>
       <c r="AA35" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -4885,7 +4885,7 @@
       </c>
       <c r="AA36" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -5022,7 +5022,7 @@
       </c>
       <c r="AA37" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -5159,7 +5159,7 @@
       </c>
       <c r="AA38" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -5296,7 +5296,7 @@
       </c>
       <c r="AA39" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -5433,7 +5433,7 @@
       </c>
       <c r="AA40" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -5570,7 +5570,7 @@
       </c>
       <c r="AA41" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -5707,7 +5707,7 @@
       </c>
       <c r="AA42" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -5834,7 +5834,7 @@
       </c>
       <c r="AA43" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -5961,7 +5961,7 @@
       </c>
       <c r="AA44" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -6088,7 +6088,7 @@
       </c>
       <c r="AA45" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -6215,7 +6215,7 @@
       </c>
       <c r="AA46" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -6342,7 +6342,7 @@
       </c>
       <c r="AA47" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -6459,7 +6459,7 @@
       </c>
       <c r="AA48" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -6591,7 +6591,7 @@
       </c>
       <c r="AA49" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -6713,7 +6713,7 @@
       </c>
       <c r="AA50" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -6845,7 +6845,7 @@
       </c>
       <c r="AA51" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -6977,7 +6977,7 @@
       </c>
       <c r="AA52" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -7114,7 +7114,7 @@
       </c>
       <c r="AA53" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="AA54" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -7388,7 +7388,7 @@
       </c>
       <c r="AA55" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -7510,7 +7510,7 @@
       </c>
       <c r="AA56" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -7637,7 +7637,7 @@
       </c>
       <c r="AA57" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -7764,7 +7764,7 @@
       </c>
       <c r="AA58" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -7881,7 +7881,7 @@
       </c>
       <c r="AA59" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -7998,7 +7998,7 @@
       </c>
       <c r="AA60" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -8125,7 +8125,7 @@
       </c>
       <c r="AA61" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -8252,7 +8252,7 @@
       </c>
       <c r="AA62" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -8379,7 +8379,7 @@
       </c>
       <c r="AA63" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -8506,7 +8506,7 @@
       </c>
       <c r="AA64" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -8633,7 +8633,7 @@
       </c>
       <c r="AA65" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -8765,7 +8765,7 @@
       </c>
       <c r="AA66" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -8887,7 +8887,7 @@
       </c>
       <c r="AA67" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -9009,7 +9009,7 @@
       </c>
       <c r="AA68" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -9131,7 +9131,7 @@
       </c>
       <c r="AA69" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AA70" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -9370,7 +9370,7 @@
       </c>
       <c r="AA71" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -9492,7 +9492,7 @@
       </c>
       <c r="AA72" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -9614,7 +9614,7 @@
       </c>
       <c r="AA73" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -9736,7 +9736,7 @@
       </c>
       <c r="AA74" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -9858,7 +9858,7 @@
       </c>
       <c r="AA75" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="AA76" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -10102,7 +10102,7 @@
       </c>
       <c r="AA77" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -10224,7 +10224,7 @@
       </c>
       <c r="AA78" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -10351,7 +10351,7 @@
       </c>
       <c r="AA79" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -10468,7 +10468,7 @@
       </c>
       <c r="AA80" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="AA81" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -10702,7 +10702,7 @@
       </c>
       <c r="AA82" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -10819,7 +10819,7 @@
       </c>
       <c r="AA83" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -10946,7 +10946,7 @@
       </c>
       <c r="AA84" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -11063,7 +11063,7 @@
       </c>
       <c r="AA85" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -11180,7 +11180,7 @@
       </c>
       <c r="AA86" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -11307,7 +11307,7 @@
       </c>
       <c r="AA87" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -11434,7 +11434,7 @@
       </c>
       <c r="AA88" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -11561,7 +11561,7 @@
       </c>
       <c r="AA89" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -11688,7 +11688,7 @@
       </c>
       <c r="AA90" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -11815,7 +11815,7 @@
       </c>
       <c r="AA91" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -11942,7 +11942,7 @@
       </c>
       <c r="AA92" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -12069,7 +12069,7 @@
       </c>
       <c r="AA93" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -12196,7 +12196,7 @@
       </c>
       <c r="AA94" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -12323,7 +12323,7 @@
       </c>
       <c r="AA95" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -12440,7 +12440,7 @@
       </c>
       <c r="AA96" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -12557,7 +12557,7 @@
       </c>
       <c r="AA97" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -12674,7 +12674,7 @@
       </c>
       <c r="AA98" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -12791,7 +12791,7 @@
       </c>
       <c r="AA99" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -12908,7 +12908,7 @@
       </c>
       <c r="AA100" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -13025,7 +13025,7 @@
       </c>
       <c r="AA101" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -13152,7 +13152,7 @@
       </c>
       <c r="AA102" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -13279,7 +13279,7 @@
       </c>
       <c r="AA103" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -13396,7 +13396,7 @@
       </c>
       <c r="AA104" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -13528,7 +13528,7 @@
       </c>
       <c r="AA105" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -13660,7 +13660,7 @@
       </c>
       <c r="AA106" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -13792,7 +13792,7 @@
       </c>
       <c r="AA107" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -13924,7 +13924,7 @@
       </c>
       <c r="AA108" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -14051,7 +14051,7 @@
       </c>
       <c r="AA109" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -14178,7 +14178,7 @@
       </c>
       <c r="AA110" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -14305,7 +14305,7 @@
       </c>
       <c r="AA111" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -14432,7 +14432,7 @@
       </c>
       <c r="AA112" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -14559,7 +14559,7 @@
       </c>
       <c r="AA113" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -14686,7 +14686,7 @@
       </c>
       <c r="AA114" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -14803,7 +14803,7 @@
       </c>
       <c r="AA115" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -14920,7 +14920,7 @@
       </c>
       <c r="AA116" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -15042,7 +15042,7 @@
       </c>
       <c r="AA117" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -15169,7 +15169,7 @@
       </c>
       <c r="AA118" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -15291,7 +15291,7 @@
       </c>
       <c r="AA119" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -15423,7 +15423,7 @@
       </c>
       <c r="AA120" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -15550,7 +15550,7 @@
       </c>
       <c r="AA121" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -15672,7 +15672,7 @@
       </c>
       <c r="AA122" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -15794,7 +15794,7 @@
       </c>
       <c r="AA123" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -15911,7 +15911,7 @@
       </c>
       <c r="AA124" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -16028,7 +16028,7 @@
       </c>
       <c r="AA125" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -16145,7 +16145,7 @@
       </c>
       <c r="AA126" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -16262,7 +16262,7 @@
       </c>
       <c r="AA127" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -16379,7 +16379,7 @@
       </c>
       <c r="AA128" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -16496,7 +16496,7 @@
       </c>
       <c r="AA129" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -16623,7 +16623,7 @@
       </c>
       <c r="AA130" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -16750,7 +16750,7 @@
       </c>
       <c r="AA131" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -16877,7 +16877,7 @@
       </c>
       <c r="AA132" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -17009,7 +17009,7 @@
       </c>
       <c r="AA133" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -17126,7 +17126,7 @@
       </c>
       <c r="AA134" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -17253,7 +17253,7 @@
       </c>
       <c r="AA135" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -17370,7 +17370,7 @@
       </c>
       <c r="AA136" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -17502,7 +17502,7 @@
       </c>
       <c r="AA137" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -17639,7 +17639,7 @@
       </c>
       <c r="AA138" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -17776,7 +17776,7 @@
       </c>
       <c r="AA139" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -17913,7 +17913,7 @@
       </c>
       <c r="AA140" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -18050,7 +18050,7 @@
       </c>
       <c r="AA141" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -18187,7 +18187,7 @@
       </c>
       <c r="AA142" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -18324,7 +18324,7 @@
       </c>
       <c r="AA143" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -18461,7 +18461,7 @@
       </c>
       <c r="AA144" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -18598,7 +18598,7 @@
       </c>
       <c r="AA145" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -18725,7 +18725,7 @@
       </c>
       <c r="AA146" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -18852,7 +18852,7 @@
       </c>
       <c r="AA147" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -18984,7 +18984,7 @@
       </c>
       <c r="AA148" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -19116,7 +19116,7 @@
       </c>
       <c r="AA149" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -19253,7 +19253,7 @@
       </c>
       <c r="AA150" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -19390,7 +19390,7 @@
       </c>
       <c r="AA151" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -19527,7 +19527,7 @@
       </c>
       <c r="AA152" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -19664,7 +19664,7 @@
       </c>
       <c r="AA153" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -19791,7 +19791,7 @@
       </c>
       <c r="AA154" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -19918,7 +19918,7 @@
       </c>
       <c r="AA155" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -20045,7 +20045,7 @@
       </c>
       <c r="AA156" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -20172,7 +20172,7 @@
       </c>
       <c r="AA157" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -20299,7 +20299,7 @@
       </c>
       <c r="AA158" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -20426,7 +20426,7 @@
       </c>
       <c r="AA159" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -20553,7 +20553,7 @@
       </c>
       <c r="AA160" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -20690,7 +20690,7 @@
       </c>
       <c r="AA161" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -20827,7 +20827,7 @@
       </c>
       <c r="AA162" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -20964,7 +20964,7 @@
       </c>
       <c r="AA163" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -21101,7 +21101,7 @@
       </c>
       <c r="AA164" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -21238,7 +21238,7 @@
       </c>
       <c r="AA165" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -21375,7 +21375,7 @@
       </c>
       <c r="AA166" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -21507,7 +21507,7 @@
       </c>
       <c r="AA167" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -21639,7 +21639,7 @@
       </c>
       <c r="AA168" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -21776,7 +21776,7 @@
       </c>
       <c r="AA169" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -21913,7 +21913,7 @@
       </c>
       <c r="AA170" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -22040,7 +22040,7 @@
       </c>
       <c r="AA171" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -22167,7 +22167,7 @@
       </c>
       <c r="AA172" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -22294,7 +22294,7 @@
       </c>
       <c r="AA173" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -22421,7 +22421,7 @@
       </c>
       <c r="AA174" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -22543,7 +22543,7 @@
       </c>
       <c r="AA175" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -22665,7 +22665,7 @@
       </c>
       <c r="AA176" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -22787,7 +22787,7 @@
       </c>
       <c r="AA177" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -22909,7 +22909,7 @@
       </c>
       <c r="AA178" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -23031,7 +23031,7 @@
       </c>
       <c r="AA179" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -23153,7 +23153,7 @@
       </c>
       <c r="AA180" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -23275,7 +23275,7 @@
       </c>
       <c r="AA181" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -23397,7 +23397,7 @@
       </c>
       <c r="AA182" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -23519,7 +23519,7 @@
       </c>
       <c r="AA183" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -23646,7 +23646,7 @@
       </c>
       <c r="AA184" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -23773,7 +23773,7 @@
       </c>
       <c r="AA185" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -23900,7 +23900,7 @@
       </c>
       <c r="AA186" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -24022,7 +24022,7 @@
       </c>
       <c r="AA187" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -24159,7 +24159,7 @@
       </c>
       <c r="AA188" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -24296,7 +24296,7 @@
       </c>
       <c r="AA189" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -24433,7 +24433,7 @@
       </c>
       <c r="AA190" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -24565,7 +24565,7 @@
       </c>
       <c r="AA191" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -24697,7 +24697,7 @@
       </c>
       <c r="AA192" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -24829,7 +24829,7 @@
       </c>
       <c r="AA193" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -24961,7 +24961,7 @@
       </c>
       <c r="AA194" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -25093,7 +25093,7 @@
       </c>
       <c r="AA195" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -25225,7 +25225,7 @@
       </c>
       <c r="AA196" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -25357,7 +25357,7 @@
       </c>
       <c r="AA197" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -25489,7 +25489,7 @@
       </c>
       <c r="AA198" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -25621,7 +25621,7 @@
       </c>
       <c r="AA199" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -25743,7 +25743,7 @@
       </c>
       <c r="AA200" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -25870,7 +25870,7 @@
       </c>
       <c r="AA201" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -25997,7 +25997,7 @@
       </c>
       <c r="AA202" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -26124,7 +26124,7 @@
       </c>
       <c r="AA203" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -26251,7 +26251,7 @@
       </c>
       <c r="AA204" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -26373,7 +26373,7 @@
       </c>
       <c r="AA205" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -26495,7 +26495,7 @@
       </c>
       <c r="AA206" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -26617,7 +26617,7 @@
       </c>
       <c r="AA207" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -26739,7 +26739,7 @@
       </c>
       <c r="AA208" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -26861,7 +26861,7 @@
       </c>
       <c r="AA209" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -26983,7 +26983,7 @@
       </c>
       <c r="AA210" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -27105,7 +27105,7 @@
       </c>
       <c r="AA211" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -27227,7 +27227,7 @@
       </c>
       <c r="AA212" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -27349,7 +27349,7 @@
       </c>
       <c r="AA213" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -27471,7 +27471,7 @@
       </c>
       <c r="AA214" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -27593,7 +27593,7 @@
       </c>
       <c r="AA215" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -27715,7 +27715,7 @@
       </c>
       <c r="AA216" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -27847,7 +27847,7 @@
       </c>
       <c r="AA217" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -27969,7 +27969,7 @@
       </c>
       <c r="AA218" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -28101,7 +28101,7 @@
       </c>
       <c r="AA219" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -28233,7 +28233,7 @@
       </c>
       <c r="AA220" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -28365,7 +28365,7 @@
       </c>
       <c r="AA221" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -28497,7 +28497,7 @@
       </c>
       <c r="AA222" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -28629,7 +28629,7 @@
       </c>
       <c r="AA223" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -28761,7 +28761,7 @@
       </c>
       <c r="AA224" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -28893,7 +28893,7 @@
       </c>
       <c r="AA225" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -29025,7 +29025,7 @@
       </c>
       <c r="AA226" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -29147,7 +29147,7 @@
       </c>
       <c r="AA227" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -29269,7 +29269,7 @@
       </c>
       <c r="AA228" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -29391,7 +29391,7 @@
       </c>
       <c r="AA229" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -29523,7 +29523,7 @@
       </c>
       <c r="AA230" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -29655,7 +29655,7 @@
       </c>
       <c r="AA231" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -29787,7 +29787,7 @@
       </c>
       <c r="AA232" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -29919,7 +29919,7 @@
       </c>
       <c r="AA233" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -30051,7 +30051,7 @@
       </c>
       <c r="AA234" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -30183,7 +30183,7 @@
       </c>
       <c r="AA235" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -30315,7 +30315,7 @@
       </c>
       <c r="AA236" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -30447,7 +30447,7 @@
       </c>
       <c r="AA237" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -30579,7 +30579,7 @@
       </c>
       <c r="AA238" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -30711,7 +30711,7 @@
       </c>
       <c r="AA239" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -30843,7 +30843,7 @@
       </c>
       <c r="AA240" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -30975,7 +30975,7 @@
       </c>
       <c r="AA241" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -31107,7 +31107,7 @@
       </c>
       <c r="AA242" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -31239,7 +31239,7 @@
       </c>
       <c r="AA243" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -31371,7 +31371,7 @@
       </c>
       <c r="AA244" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -31503,7 +31503,7 @@
       </c>
       <c r="AA245" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -31635,7 +31635,7 @@
       </c>
       <c r="AA246" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -31762,7 +31762,7 @@
       </c>
       <c r="AA247" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -31889,7 +31889,7 @@
       </c>
       <c r="AA248" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -32016,7 +32016,7 @@
       </c>
       <c r="AA249" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -32143,7 +32143,7 @@
       </c>
       <c r="AA250" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -32270,7 +32270,7 @@
       </c>
       <c r="AA251" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -32402,7 +32402,7 @@
       </c>
       <c r="AA252" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -32534,7 +32534,7 @@
       </c>
       <c r="AA253" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -32666,7 +32666,7 @@
       </c>
       <c r="AA254" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -32798,7 +32798,7 @@
       </c>
       <c r="AA255" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -32930,7 +32930,7 @@
       </c>
       <c r="AA256" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -33062,7 +33062,7 @@
       </c>
       <c r="AA257" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -33194,7 +33194,7 @@
       </c>
       <c r="AA258" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -33326,7 +33326,7 @@
       </c>
       <c r="AA259" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -33458,7 +33458,7 @@
       </c>
       <c r="AA260" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -33590,7 +33590,7 @@
       </c>
       <c r="AA261" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -33722,7 +33722,7 @@
       </c>
       <c r="AA262" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -33854,7 +33854,7 @@
       </c>
       <c r="AA263" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -33986,7 +33986,7 @@
       </c>
       <c r="AA264" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -34118,7 +34118,7 @@
       </c>
       <c r="AA265" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -34250,7 +34250,7 @@
       </c>
       <c r="AA266" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -34382,7 +34382,7 @@
       </c>
       <c r="AA267" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -34514,7 +34514,7 @@
       </c>
       <c r="AA268" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
@@ -34646,14 +34646,14 @@
       </c>
       <c r="AA269" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="270">
       <c r="A270" s="0" t="inlineStr">
         <is>
-          <t>18824</t>
+          <t>18831</t>
         </is>
       </c>
       <c r="B270" s="0" t="inlineStr">
@@ -34663,7 +34663,7 @@
       </c>
       <c r="C270" s="0" t="inlineStr">
         <is>
-          <t>VAU118970</t>
+          <t>VAU118978</t>
         </is>
       </c>
       <c r="D270" s="0" t="inlineStr">
@@ -34683,12 +34683,12 @@
       </c>
       <c r="G270" s="0" t="inlineStr">
         <is>
-          <t>006614</t>
+          <t>010136</t>
         </is>
       </c>
       <c r="H270" s="0" t="inlineStr">
         <is>
-          <t>Scala Montabaur, Chlebowski</t>
+          <t>Naci Agcagül, Scala Montabaur</t>
         </is>
       </c>
       <c r="K270" s="0" t="inlineStr">
@@ -34703,7 +34703,7 @@
       </c>
       <c r="M270" s="0" t="inlineStr">
         <is>
-          <t>VAU118970</t>
+          <t>VAU118978</t>
         </is>
       </c>
       <c r="N270" s="0" t="inlineStr">
@@ -34743,12 +34743,12 @@
       </c>
       <c r="W270" s="0" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="X270" s="0" t="inlineStr">
         <is>
-          <t>[ ** 1 (KO_1) (LS_1) (RE_0) (LA_1) (RB_0) (AB_0) ** Uwe Chlebowski 0160 46 599 84 ** ]</t>
+          <t>[ ** 1 (KO_0) (LS_0) (RE_0) (LA_0) (RB_1) (AB_0) ** Anlieferung durch WWB / Freitag ** ]</t>
         </is>
       </c>
       <c r="Y270" s="0" t="inlineStr">
@@ -34763,7 +34763,7 @@
       </c>
       <c r="AA270" s="0" t="inlineStr">
         <is>
-          <t>11.02.2026 15:57:45:990</t>
+          <t>11.02.2026 16:47:01:620</t>
         </is>
       </c>
     </row>

</xml_diff>